<commit_message>
Fixed duplicate frame bug for FLX
</commit_message>
<xml_diff>
--- a/image manifest.xlsx
+++ b/image manifest.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\Github\CS-Graphics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6EEC027-C783-4DB6-860C-107F07F3C5E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD999E39-EF47-4172-920C-DA109F2DBD4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{620D0F7A-D0D3-4EA0-8A4D-C0BB25CE06A6}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="4" r:id="rId3"/>
+    <pivotCache cacheId="0" r:id="rId3"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -4561,7 +4561,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
@@ -4569,7 +4569,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -19731,7 +19730,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FA313DB3-B760-4691-87E1-B5DF4E7F9B43}" name="PivotTable3" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FA313DB3-B760-4691-87E1-B5DF4E7F9B43}" name="PivotTable3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:C9" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="11">
     <pivotField showAll="0"/>
@@ -49469,7 +49468,7 @@
         <v>1132</v>
       </c>
       <c r="E906">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F906" t="s">
         <v>914</v>
@@ -49501,7 +49500,7 @@
         <v>1132</v>
       </c>
       <c r="E907">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F907" t="s">
         <v>914</v>
@@ -49533,7 +49532,7 @@
         <v>1132</v>
       </c>
       <c r="E908">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F908" t="s">
         <v>914</v>
@@ -49565,7 +49564,7 @@
         <v>1132</v>
       </c>
       <c r="E909">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F909" t="s">
         <v>914</v>
@@ -49597,7 +49596,7 @@
         <v>1132</v>
       </c>
       <c r="E910">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F910" t="s">
         <v>914</v>
@@ -49629,7 +49628,7 @@
         <v>1132</v>
       </c>
       <c r="E911">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F911" t="s">
         <v>914</v>
@@ -49661,7 +49660,7 @@
         <v>1132</v>
       </c>
       <c r="E912">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F912" t="s">
         <v>914</v>
@@ -49693,7 +49692,7 @@
         <v>1132</v>
       </c>
       <c r="E913">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F913" t="s">
         <v>914</v>
@@ -49725,7 +49724,7 @@
         <v>1132</v>
       </c>
       <c r="E914">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F914" t="s">
         <v>914</v>
@@ -49757,7 +49756,7 @@
         <v>1132</v>
       </c>
       <c r="E915">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F915" t="s">
         <v>914</v>
@@ -49789,7 +49788,7 @@
         <v>1132</v>
       </c>
       <c r="E916">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F916" t="s">
         <v>914</v>
@@ -49821,7 +49820,7 @@
         <v>1132</v>
       </c>
       <c r="E917">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F917" t="s">
         <v>914</v>
@@ -49853,7 +49852,7 @@
         <v>1132</v>
       </c>
       <c r="E918">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F918" t="s">
         <v>914</v>
@@ -49885,7 +49884,7 @@
         <v>1132</v>
       </c>
       <c r="E919">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F919" t="s">
         <v>914</v>
@@ -49917,7 +49916,7 @@
         <v>1132</v>
       </c>
       <c r="E920">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F920" t="s">
         <v>914</v>
@@ -49949,7 +49948,7 @@
         <v>1132</v>
       </c>
       <c r="E921">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F921" t="s">
         <v>914</v>
@@ -49981,7 +49980,7 @@
         <v>1132</v>
       </c>
       <c r="E922">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F922" t="s">
         <v>914</v>
@@ -50013,7 +50012,7 @@
         <v>1132</v>
       </c>
       <c r="E923">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F923" t="s">
         <v>914</v>
@@ -50045,7 +50044,7 @@
         <v>1132</v>
       </c>
       <c r="E924">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F924" t="s">
         <v>914</v>
@@ -50077,7 +50076,7 @@
         <v>1132</v>
       </c>
       <c r="E925">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F925" t="s">
         <v>914</v>
@@ -50109,7 +50108,7 @@
         <v>1132</v>
       </c>
       <c r="E926">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F926" t="s">
         <v>914</v>
@@ -50141,7 +50140,7 @@
         <v>1132</v>
       </c>
       <c r="E927">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F927" t="s">
         <v>914</v>
@@ -50173,7 +50172,7 @@
         <v>1132</v>
       </c>
       <c r="E928">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F928" t="s">
         <v>914</v>
@@ -50205,7 +50204,7 @@
         <v>1132</v>
       </c>
       <c r="E929">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F929" t="s">
         <v>914</v>
@@ -50237,7 +50236,7 @@
         <v>1132</v>
       </c>
       <c r="E930">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F930" t="s">
         <v>914</v>
@@ -50269,7 +50268,7 @@
         <v>1132</v>
       </c>
       <c r="E931">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F931" t="s">
         <v>914</v>
@@ -50301,7 +50300,7 @@
         <v>1132</v>
       </c>
       <c r="E932">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F932" t="s">
         <v>914</v>
@@ -50333,7 +50332,7 @@
         <v>1132</v>
       </c>
       <c r="E933">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F933" t="s">
         <v>914</v>
@@ -50365,7 +50364,7 @@
         <v>1132</v>
       </c>
       <c r="E934">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F934" t="s">
         <v>914</v>
@@ -50397,7 +50396,7 @@
         <v>1132</v>
       </c>
       <c r="E935">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F935" t="s">
         <v>914</v>
@@ -50429,7 +50428,7 @@
         <v>1132</v>
       </c>
       <c r="E936">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F936" t="s">
         <v>914</v>
@@ -50461,7 +50460,7 @@
         <v>1132</v>
       </c>
       <c r="E937">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F937" t="s">
         <v>914</v>
@@ -50493,7 +50492,7 @@
         <v>1132</v>
       </c>
       <c r="E938">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F938" t="s">
         <v>914</v>
@@ -50525,7 +50524,7 @@
         <v>1132</v>
       </c>
       <c r="E939">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F939" t="s">
         <v>914</v>
@@ -50557,7 +50556,7 @@
         <v>1132</v>
       </c>
       <c r="E940">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F940" t="s">
         <v>914</v>
@@ -50589,7 +50588,7 @@
         <v>1132</v>
       </c>
       <c r="E941">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F941" t="s">
         <v>914</v>
@@ -50621,7 +50620,7 @@
         <v>1132</v>
       </c>
       <c r="E942">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F942" t="s">
         <v>914</v>
@@ -50653,7 +50652,7 @@
         <v>1132</v>
       </c>
       <c r="E943">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F943" t="s">
         <v>914</v>
@@ -50685,7 +50684,7 @@
         <v>1132</v>
       </c>
       <c r="E944">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F944" t="s">
         <v>914</v>
@@ -50717,7 +50716,7 @@
         <v>1132</v>
       </c>
       <c r="E945">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F945" t="s">
         <v>914</v>
@@ -50749,7 +50748,7 @@
         <v>1132</v>
       </c>
       <c r="E946">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F946" t="s">
         <v>914</v>
@@ -50781,7 +50780,7 @@
         <v>1132</v>
       </c>
       <c r="E947">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F947" t="s">
         <v>914</v>
@@ -50813,7 +50812,7 @@
         <v>1132</v>
       </c>
       <c r="E948">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F948" t="s">
         <v>914</v>
@@ -50845,7 +50844,7 @@
         <v>1132</v>
       </c>
       <c r="E949">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F949" t="s">
         <v>914</v>
@@ -50877,7 +50876,7 @@
         <v>1132</v>
       </c>
       <c r="E950">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F950" t="s">
         <v>914</v>
@@ -50909,7 +50908,7 @@
         <v>1132</v>
       </c>
       <c r="E951">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F951" t="s">
         <v>914</v>
@@ -50941,7 +50940,7 @@
         <v>1132</v>
       </c>
       <c r="E952">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F952" t="s">
         <v>914</v>
@@ -50973,7 +50972,7 @@
         <v>1132</v>
       </c>
       <c r="E953">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F953" t="s">
         <v>914</v>
@@ -51005,7 +51004,7 @@
         <v>1132</v>
       </c>
       <c r="E954">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F954" t="s">
         <v>914</v>
@@ -51037,7 +51036,7 @@
         <v>1132</v>
       </c>
       <c r="E955">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F955" t="s">
         <v>914</v>
@@ -51069,7 +51068,7 @@
         <v>1132</v>
       </c>
       <c r="E956">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F956" t="s">
         <v>914</v>
@@ -51101,7 +51100,7 @@
         <v>1132</v>
       </c>
       <c r="E957">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F957" t="s">
         <v>914</v>
@@ -51133,7 +51132,7 @@
         <v>1132</v>
       </c>
       <c r="E958">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F958" t="s">
         <v>914</v>
@@ -51165,7 +51164,7 @@
         <v>1132</v>
       </c>
       <c r="E959">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F959" t="s">
         <v>914</v>
@@ -51197,7 +51196,7 @@
         <v>1132</v>
       </c>
       <c r="E960">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F960" t="s">
         <v>914</v>
@@ -51229,7 +51228,7 @@
         <v>1132</v>
       </c>
       <c r="E961">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F961" t="s">
         <v>914</v>
@@ -51261,7 +51260,7 @@
         <v>1132</v>
       </c>
       <c r="E962">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F962" t="s">
         <v>914</v>
@@ -51293,7 +51292,7 @@
         <v>1132</v>
       </c>
       <c r="E963">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F963" t="s">
         <v>914</v>
@@ -51325,7 +51324,7 @@
         <v>1132</v>
       </c>
       <c r="E964">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F964" t="s">
         <v>914</v>
@@ -51357,7 +51356,7 @@
         <v>1132</v>
       </c>
       <c r="E965">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F965" t="s">
         <v>914</v>
@@ -51389,7 +51388,7 @@
         <v>1132</v>
       </c>
       <c r="E966">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F966" t="s">
         <v>914</v>
@@ -51421,7 +51420,7 @@
         <v>1132</v>
       </c>
       <c r="E967">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F967" t="s">
         <v>914</v>
@@ -51453,7 +51452,7 @@
         <v>1132</v>
       </c>
       <c r="E968">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F968" t="s">
         <v>914</v>
@@ -51485,7 +51484,7 @@
         <v>1132</v>
       </c>
       <c r="E969">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F969" t="s">
         <v>914</v>
@@ -51517,7 +51516,7 @@
         <v>1132</v>
       </c>
       <c r="E970">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F970" t="s">
         <v>914</v>
@@ -51549,7 +51548,7 @@
         <v>1132</v>
       </c>
       <c r="E971">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F971" t="s">
         <v>914</v>
@@ -51581,7 +51580,7 @@
         <v>1132</v>
       </c>
       <c r="E972">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F972" t="s">
         <v>914</v>
@@ -51613,7 +51612,7 @@
         <v>1132</v>
       </c>
       <c r="E973">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F973" t="s">
         <v>914</v>
@@ -51645,7 +51644,7 @@
         <v>1132</v>
       </c>
       <c r="E974">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F974" t="s">
         <v>914</v>
@@ -51677,7 +51676,7 @@
         <v>1132</v>
       </c>
       <c r="E975">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F975" t="s">
         <v>914</v>
@@ -51709,7 +51708,7 @@
         <v>1132</v>
       </c>
       <c r="E976">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F976" t="s">
         <v>914</v>
@@ -51741,7 +51740,7 @@
         <v>1132</v>
       </c>
       <c r="E977">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F977" t="s">
         <v>914</v>
@@ -51773,7 +51772,7 @@
         <v>1132</v>
       </c>
       <c r="E978">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F978" t="s">
         <v>914</v>
@@ -51805,7 +51804,7 @@
         <v>1132</v>
       </c>
       <c r="E979">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F979" t="s">
         <v>914</v>
@@ -51837,7 +51836,7 @@
         <v>1132</v>
       </c>
       <c r="E980">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F980" t="s">
         <v>914</v>
@@ -51869,7 +51868,7 @@
         <v>1132</v>
       </c>
       <c r="E981">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F981" t="s">
         <v>914</v>
@@ -51901,7 +51900,7 @@
         <v>1132</v>
       </c>
       <c r="E982">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F982" t="s">
         <v>914</v>
@@ -51933,7 +51932,7 @@
         <v>1132</v>
       </c>
       <c r="E983">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F983" t="s">
         <v>914</v>
@@ -51965,7 +51964,7 @@
         <v>1132</v>
       </c>
       <c r="E984">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F984" t="s">
         <v>914</v>
@@ -51997,7 +51996,7 @@
         <v>1132</v>
       </c>
       <c r="E985">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F985" t="s">
         <v>914</v>
@@ -52029,7 +52028,7 @@
         <v>1132</v>
       </c>
       <c r="E986">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F986" t="s">
         <v>914</v>
@@ -52061,7 +52060,7 @@
         <v>1132</v>
       </c>
       <c r="E987">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F987" t="s">
         <v>914</v>
@@ -52093,7 +52092,7 @@
         <v>1132</v>
       </c>
       <c r="E988">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F988" t="s">
         <v>914</v>
@@ -52125,7 +52124,7 @@
         <v>1132</v>
       </c>
       <c r="E989">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F989" t="s">
         <v>914</v>
@@ -52157,7 +52156,7 @@
         <v>1132</v>
       </c>
       <c r="E990">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F990" t="s">
         <v>914</v>
@@ -52189,7 +52188,7 @@
         <v>1132</v>
       </c>
       <c r="E991">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F991" t="s">
         <v>914</v>
@@ -52221,7 +52220,7 @@
         <v>1132</v>
       </c>
       <c r="E992">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F992" t="s">
         <v>914</v>
@@ -52253,7 +52252,7 @@
         <v>1132</v>
       </c>
       <c r="E993">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F993" t="s">
         <v>914</v>
@@ -52285,7 +52284,7 @@
         <v>1132</v>
       </c>
       <c r="E994">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F994" t="s">
         <v>914</v>
@@ -52317,7 +52316,7 @@
         <v>1132</v>
       </c>
       <c r="E995">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F995" t="s">
         <v>914</v>
@@ -52349,7 +52348,7 @@
         <v>1132</v>
       </c>
       <c r="E996">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F996" t="s">
         <v>914</v>
@@ -52381,7 +52380,7 @@
         <v>1132</v>
       </c>
       <c r="E997">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F997" t="s">
         <v>914</v>
@@ -52413,7 +52412,7 @@
         <v>1132</v>
       </c>
       <c r="E998">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F998" t="s">
         <v>914</v>
@@ -52445,7 +52444,7 @@
         <v>1132</v>
       </c>
       <c r="E999">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F999" t="s">
         <v>914</v>
@@ -52477,7 +52476,7 @@
         <v>1132</v>
       </c>
       <c r="E1000">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1000" t="s">
         <v>914</v>
@@ -52509,7 +52508,7 @@
         <v>1132</v>
       </c>
       <c r="E1001">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1001" t="s">
         <v>914</v>
@@ -52541,7 +52540,7 @@
         <v>1132</v>
       </c>
       <c r="E1002">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1002" t="s">
         <v>914</v>
@@ -52573,7 +52572,7 @@
         <v>1132</v>
       </c>
       <c r="E1003">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1003" t="s">
         <v>914</v>
@@ -52605,7 +52604,7 @@
         <v>1132</v>
       </c>
       <c r="E1004">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1004" t="s">
         <v>914</v>
@@ -52637,7 +52636,7 @@
         <v>1132</v>
       </c>
       <c r="E1005">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1005" t="s">
         <v>914</v>
@@ -52669,7 +52668,7 @@
         <v>1132</v>
       </c>
       <c r="E1006">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1006" t="s">
         <v>914</v>
@@ -52701,7 +52700,7 @@
         <v>1132</v>
       </c>
       <c r="E1007">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="F1007" t="s">
         <v>914</v>
@@ -52733,7 +52732,7 @@
         <v>1132</v>
       </c>
       <c r="E1008">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1008" t="s">
         <v>914</v>
@@ -52765,7 +52764,7 @@
         <v>1132</v>
       </c>
       <c r="E1009">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1009" t="s">
         <v>914</v>
@@ -52797,7 +52796,7 @@
         <v>1132</v>
       </c>
       <c r="E1010">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1010" t="s">
         <v>914</v>
@@ -52829,7 +52828,7 @@
         <v>1132</v>
       </c>
       <c r="E1011">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1011" t="s">
         <v>914</v>
@@ -52861,7 +52860,7 @@
         <v>1132</v>
       </c>
       <c r="E1012">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1012" t="s">
         <v>914</v>
@@ -52893,7 +52892,7 @@
         <v>1132</v>
       </c>
       <c r="E1013">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1013" t="s">
         <v>914</v>
@@ -52925,7 +52924,7 @@
         <v>1132</v>
       </c>
       <c r="E1014">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1014" t="s">
         <v>914</v>
@@ -52957,7 +52956,7 @@
         <v>1132</v>
       </c>
       <c r="E1015">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1015" t="s">
         <v>914</v>
@@ -52989,7 +52988,7 @@
         <v>1132</v>
       </c>
       <c r="E1016">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1016" t="s">
         <v>914</v>
@@ -53021,7 +53020,7 @@
         <v>1132</v>
       </c>
       <c r="E1017">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1017" t="s">
         <v>914</v>
@@ -53053,7 +53052,7 @@
         <v>1132</v>
       </c>
       <c r="E1018">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1018" t="s">
         <v>914</v>
@@ -53085,7 +53084,7 @@
         <v>1132</v>
       </c>
       <c r="E1019">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1019" t="s">
         <v>914</v>
@@ -53117,7 +53116,7 @@
         <v>1132</v>
       </c>
       <c r="E1020">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1020" t="s">
         <v>914</v>
@@ -53149,7 +53148,7 @@
         <v>1132</v>
       </c>
       <c r="E1021">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1021" t="s">
         <v>914</v>
@@ -53181,7 +53180,7 @@
         <v>1132</v>
       </c>
       <c r="E1022">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1022" t="s">
         <v>914</v>
@@ -53213,7 +53212,7 @@
         <v>1132</v>
       </c>
       <c r="E1023">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1023" t="s">
         <v>914</v>
@@ -53245,7 +53244,7 @@
         <v>1132</v>
       </c>
       <c r="E1024">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1024" t="s">
         <v>914</v>
@@ -53277,7 +53276,7 @@
         <v>1132</v>
       </c>
       <c r="E1025">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1025" t="s">
         <v>914</v>
@@ -53309,7 +53308,7 @@
         <v>1132</v>
       </c>
       <c r="E1026">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1026" t="s">
         <v>914</v>
@@ -53341,7 +53340,7 @@
         <v>1132</v>
       </c>
       <c r="E1027">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1027" t="s">
         <v>914</v>
@@ -53373,7 +53372,7 @@
         <v>1132</v>
       </c>
       <c r="E1028">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1028" t="s">
         <v>914</v>
@@ -53405,7 +53404,7 @@
         <v>1132</v>
       </c>
       <c r="E1029">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1029" t="s">
         <v>914</v>
@@ -53437,7 +53436,7 @@
         <v>1132</v>
       </c>
       <c r="E1030">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1030" t="s">
         <v>914</v>
@@ -53469,7 +53468,7 @@
         <v>1132</v>
       </c>
       <c r="E1031">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1031" t="s">
         <v>914</v>
@@ -53501,7 +53500,7 @@
         <v>1132</v>
       </c>
       <c r="E1032">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F1032" t="s">
         <v>914</v>
@@ -53533,7 +53532,7 @@
         <v>1132</v>
       </c>
       <c r="E1033">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F1033" t="s">
         <v>914</v>
@@ -53565,7 +53564,7 @@
         <v>1132</v>
       </c>
       <c r="E1034">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F1034" t="s">
         <v>914</v>
@@ -53597,7 +53596,7 @@
         <v>1132</v>
       </c>
       <c r="E1035">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F1035" t="s">
         <v>914</v>
@@ -53629,7 +53628,7 @@
         <v>1132</v>
       </c>
       <c r="E1036">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F1036" t="s">
         <v>914</v>
@@ -53661,7 +53660,7 @@
         <v>1132</v>
       </c>
       <c r="E1037">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F1037" t="s">
         <v>914</v>
@@ -53693,7 +53692,7 @@
         <v>1132</v>
       </c>
       <c r="E1038">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F1038" t="s">
         <v>914</v>
@@ -53725,7 +53724,7 @@
         <v>1132</v>
       </c>
       <c r="E1039">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F1039" t="s">
         <v>914</v>
@@ -53757,7 +53756,7 @@
         <v>1132</v>
       </c>
       <c r="E1040">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F1040" t="s">
         <v>914</v>
@@ -53789,7 +53788,7 @@
         <v>1132</v>
       </c>
       <c r="E1041">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F1041" t="s">
         <v>914</v>
@@ -53821,7 +53820,7 @@
         <v>1132</v>
       </c>
       <c r="E1042">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F1042" t="s">
         <v>914</v>
@@ -53853,7 +53852,7 @@
         <v>1132</v>
       </c>
       <c r="E1043">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F1043" t="s">
         <v>914</v>
@@ -53885,7 +53884,7 @@
         <v>1132</v>
       </c>
       <c r="E1044">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F1044" t="s">
         <v>914</v>
@@ -53917,7 +53916,7 @@
         <v>1132</v>
       </c>
       <c r="E1045">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F1045" t="s">
         <v>914</v>
@@ -53949,7 +53948,7 @@
         <v>1132</v>
       </c>
       <c r="E1046">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F1046" t="s">
         <v>914</v>
@@ -53981,7 +53980,7 @@
         <v>1132</v>
       </c>
       <c r="E1047">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F1047" t="s">
         <v>914</v>
@@ -54013,7 +54012,7 @@
         <v>1132</v>
       </c>
       <c r="E1048">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F1048" t="s">
         <v>914</v>
@@ -54045,7 +54044,7 @@
         <v>1132</v>
       </c>
       <c r="E1049">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F1049" t="s">
         <v>914</v>
@@ -54077,7 +54076,7 @@
         <v>1132</v>
       </c>
       <c r="E1050">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F1050" t="s">
         <v>914</v>
@@ -54109,7 +54108,7 @@
         <v>1132</v>
       </c>
       <c r="E1051">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F1051" t="s">
         <v>914</v>
@@ -54141,7 +54140,7 @@
         <v>1132</v>
       </c>
       <c r="E1052">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F1052" t="s">
         <v>914</v>
@@ -54173,7 +54172,7 @@
         <v>1132</v>
       </c>
       <c r="E1053">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F1053" t="s">
         <v>914</v>
@@ -54205,7 +54204,7 @@
         <v>1132</v>
       </c>
       <c r="E1054">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F1054" t="s">
         <v>914</v>
@@ -54251,7 +54250,7 @@
         <v>1132</v>
       </c>
       <c r="E1056">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1056" t="s">
         <v>914</v>
@@ -54297,7 +54296,7 @@
         <v>1132</v>
       </c>
       <c r="E1058">
-        <v>1801</v>
+        <v>1800</v>
       </c>
       <c r="F1058" t="s">
         <v>914</v>
@@ -54329,7 +54328,7 @@
         <v>1132</v>
       </c>
       <c r="E1059">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F1059" t="s">
         <v>914</v>
@@ -54361,7 +54360,7 @@
         <v>1132</v>
       </c>
       <c r="E1060">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F1060" t="s">
         <v>914</v>
@@ -54407,7 +54406,7 @@
         <v>1132</v>
       </c>
       <c r="E1062">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F1062" t="s">
         <v>914</v>
@@ -54439,7 +54438,7 @@
         <v>1132</v>
       </c>
       <c r="E1063">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F1063" t="s">
         <v>914</v>
@@ -54471,7 +54470,7 @@
         <v>1132</v>
       </c>
       <c r="E1064">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F1064" t="s">
         <v>914</v>
@@ -54503,7 +54502,7 @@
         <v>1132</v>
       </c>
       <c r="E1065">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F1065" t="s">
         <v>914</v>
@@ -54535,7 +54534,7 @@
         <v>1132</v>
       </c>
       <c r="E1066">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F1066" t="s">
         <v>914</v>
@@ -54567,7 +54566,7 @@
         <v>1132</v>
       </c>
       <c r="E1067">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F1067" t="s">
         <v>914</v>
@@ -54599,7 +54598,7 @@
         <v>1132</v>
       </c>
       <c r="E1068">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F1068" t="s">
         <v>914</v>
@@ -54631,7 +54630,7 @@
         <v>1132</v>
       </c>
       <c r="E1069">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F1069" t="s">
         <v>914</v>
@@ -54663,7 +54662,7 @@
         <v>1132</v>
       </c>
       <c r="E1070">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F1070" t="s">
         <v>914</v>
@@ -54759,7 +54758,7 @@
         <v>1132</v>
       </c>
       <c r="E1073">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F1073" t="s">
         <v>914</v>
@@ -54791,7 +54790,7 @@
         <v>1132</v>
       </c>
       <c r="E1074">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F1074" t="s">
         <v>914</v>
@@ -54823,7 +54822,7 @@
         <v>1132</v>
       </c>
       <c r="E1075">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F1075" t="s">
         <v>914</v>
@@ -54855,7 +54854,7 @@
         <v>1132</v>
       </c>
       <c r="E1076">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F1076" t="s">
         <v>914</v>
@@ -54887,7 +54886,7 @@
         <v>1132</v>
       </c>
       <c r="E1077">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F1077" t="s">
         <v>914</v>
@@ -54919,7 +54918,7 @@
         <v>1132</v>
       </c>
       <c r="E1078">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F1078" t="s">
         <v>914</v>
@@ -54951,7 +54950,7 @@
         <v>1132</v>
       </c>
       <c r="E1079">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F1079" t="s">
         <v>914</v>
@@ -54983,7 +54982,7 @@
         <v>1132</v>
       </c>
       <c r="E1080">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F1080" t="s">
         <v>914</v>
@@ -55015,7 +55014,7 @@
         <v>1132</v>
       </c>
       <c r="E1081">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F1081" t="s">
         <v>914</v>
@@ -55047,7 +55046,7 @@
         <v>1132</v>
       </c>
       <c r="E1082">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F1082" t="s">
         <v>914</v>
@@ -55079,7 +55078,7 @@
         <v>1132</v>
       </c>
       <c r="E1083">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F1083" t="s">
         <v>914</v>
@@ -55111,7 +55110,7 @@
         <v>1132</v>
       </c>
       <c r="E1084">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F1084" t="s">
         <v>914</v>
@@ -55143,7 +55142,7 @@
         <v>1132</v>
       </c>
       <c r="E1085">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1085" t="s">
         <v>914</v>
@@ -55175,7 +55174,7 @@
         <v>1132</v>
       </c>
       <c r="E1086">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F1086" t="s">
         <v>914</v>
@@ -55207,7 +55206,7 @@
         <v>1132</v>
       </c>
       <c r="E1087">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F1087" t="s">
         <v>914</v>
@@ -55239,7 +55238,7 @@
         <v>1132</v>
       </c>
       <c r="E1088">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F1088" t="s">
         <v>914</v>
@@ -55271,7 +55270,7 @@
         <v>1132</v>
       </c>
       <c r="E1089">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="F1089" t="s">
         <v>914</v>
@@ -55317,7 +55316,7 @@
         <v>1132</v>
       </c>
       <c r="E1091">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F1091" t="s">
         <v>914</v>
@@ -55349,7 +55348,7 @@
         <v>1132</v>
       </c>
       <c r="E1092">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F1092" t="s">
         <v>914</v>
@@ -55381,7 +55380,7 @@
         <v>1132</v>
       </c>
       <c r="E1093">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1093" t="s">
         <v>914</v>
@@ -55413,7 +55412,7 @@
         <v>1132</v>
       </c>
       <c r="E1094">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F1094" t="s">
         <v>914</v>
@@ -55445,7 +55444,7 @@
         <v>1132</v>
       </c>
       <c r="E1095">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1095" t="s">
         <v>914</v>
@@ -55477,7 +55476,7 @@
         <v>1132</v>
       </c>
       <c r="E1096">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1096" t="s">
         <v>914</v>
@@ -55509,7 +55508,7 @@
         <v>1132</v>
       </c>
       <c r="E1097">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1097" t="s">
         <v>914</v>
@@ -55541,7 +55540,7 @@
         <v>1132</v>
       </c>
       <c r="E1098">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F1098" t="s">
         <v>914</v>
@@ -55573,7 +55572,7 @@
         <v>1132</v>
       </c>
       <c r="E1099">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F1099" t="s">
         <v>914</v>
@@ -55605,7 +55604,7 @@
         <v>1132</v>
       </c>
       <c r="E1100">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F1100" t="s">
         <v>914</v>
@@ -55637,7 +55636,7 @@
         <v>1132</v>
       </c>
       <c r="E1101">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F1101" t="s">
         <v>914</v>
@@ -55669,7 +55668,7 @@
         <v>1132</v>
       </c>
       <c r="E1102">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F1102" t="s">
         <v>914</v>
@@ -55701,7 +55700,7 @@
         <v>1132</v>
       </c>
       <c r="E1103">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F1103" t="s">
         <v>914</v>
@@ -55733,7 +55732,7 @@
         <v>1132</v>
       </c>
       <c r="E1104">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F1104" t="s">
         <v>914</v>
@@ -55765,7 +55764,7 @@
         <v>1132</v>
       </c>
       <c r="E1105">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F1105" t="s">
         <v>914</v>
@@ -55797,7 +55796,7 @@
         <v>1132</v>
       </c>
       <c r="E1106">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F1106" t="s">
         <v>914</v>
@@ -55829,7 +55828,7 @@
         <v>1132</v>
       </c>
       <c r="E1107">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F1107" t="s">
         <v>914</v>
@@ -55861,7 +55860,7 @@
         <v>1132</v>
       </c>
       <c r="E1108">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F1108" t="s">
         <v>914</v>
@@ -55893,7 +55892,7 @@
         <v>1132</v>
       </c>
       <c r="E1109">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F1109" t="s">
         <v>914</v>
@@ -55925,7 +55924,7 @@
         <v>1132</v>
       </c>
       <c r="E1110">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F1110" t="s">
         <v>914</v>
@@ -55957,7 +55956,7 @@
         <v>1132</v>
       </c>
       <c r="E1111">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F1111" t="s">
         <v>914</v>
@@ -55989,7 +55988,7 @@
         <v>1132</v>
       </c>
       <c r="E1112">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F1112" t="s">
         <v>914</v>
@@ -56021,7 +56020,7 @@
         <v>1132</v>
       </c>
       <c r="E1113">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F1113" t="s">
         <v>914</v>
@@ -56053,7 +56052,7 @@
         <v>1132</v>
       </c>
       <c r="E1114">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1114" t="s">
         <v>914</v>
@@ -56085,7 +56084,7 @@
         <v>1132</v>
       </c>
       <c r="E1115">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F1115" t="s">
         <v>914</v>
@@ -56117,7 +56116,7 @@
         <v>1132</v>
       </c>
       <c r="E1116">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F1116" t="s">
         <v>914</v>
@@ -56149,7 +56148,7 @@
         <v>1132</v>
       </c>
       <c r="E1117">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F1117" t="s">
         <v>914</v>
@@ -56181,7 +56180,7 @@
         <v>1132</v>
       </c>
       <c r="E1118">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F1118" t="s">
         <v>914</v>
@@ -56213,7 +56212,7 @@
         <v>1132</v>
       </c>
       <c r="E1119">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1119" t="s">
         <v>914</v>
@@ -56245,7 +56244,7 @@
         <v>1132</v>
       </c>
       <c r="E1120">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1120" t="s">
         <v>914</v>
@@ -56277,7 +56276,7 @@
         <v>1132</v>
       </c>
       <c r="E1121">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1121" t="s">
         <v>914</v>
@@ -56309,7 +56308,7 @@
         <v>1132</v>
       </c>
       <c r="E1122">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F1122" t="s">
         <v>914</v>
@@ -56341,7 +56340,7 @@
         <v>1132</v>
       </c>
       <c r="E1123">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F1123" t="s">
         <v>914</v>
@@ -56373,7 +56372,7 @@
         <v>1132</v>
       </c>
       <c r="E1124">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F1124" t="s">
         <v>914</v>
@@ -56405,7 +56404,7 @@
         <v>1132</v>
       </c>
       <c r="E1125">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F1125" t="s">
         <v>914</v>
@@ -56437,7 +56436,7 @@
         <v>1132</v>
       </c>
       <c r="E1126">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F1126" t="s">
         <v>914</v>
@@ -56469,7 +56468,7 @@
         <v>1132</v>
       </c>
       <c r="E1127">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F1127" t="s">
         <v>914</v>
@@ -56501,7 +56500,7 @@
         <v>1132</v>
       </c>
       <c r="E1128">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1128" t="s">
         <v>914</v>
@@ -56533,7 +56532,7 @@
         <v>1132</v>
       </c>
       <c r="E1129">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1129" t="s">
         <v>914</v>
@@ -56579,7 +56578,7 @@
         <v>1132</v>
       </c>
       <c r="E1131">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F1131" t="s">
         <v>914</v>
@@ -56611,7 +56610,7 @@
         <v>1132</v>
       </c>
       <c r="E1132">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F1132" t="s">
         <v>914</v>
@@ -56657,7 +56656,7 @@
         <v>1132</v>
       </c>
       <c r="E1134">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1134" t="s">
         <v>914</v>
@@ -56689,7 +56688,7 @@
         <v>1132</v>
       </c>
       <c r="E1135">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F1135" t="s">
         <v>914</v>
@@ -56785,7 +56784,7 @@
         <v>1132</v>
       </c>
       <c r="E1138">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="F1138" t="s">
         <v>914</v>
@@ -56817,7 +56816,7 @@
         <v>1132</v>
       </c>
       <c r="E1139">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F1139" t="s">
         <v>914</v>
@@ -56849,7 +56848,7 @@
         <v>1132</v>
       </c>
       <c r="E1140">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F1140" t="s">
         <v>914</v>
@@ -56881,7 +56880,7 @@
         <v>1132</v>
       </c>
       <c r="E1141">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F1141" t="s">
         <v>914</v>
@@ -56913,7 +56912,7 @@
         <v>1132</v>
       </c>
       <c r="E1142">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F1142" t="s">
         <v>914</v>
@@ -56945,7 +56944,7 @@
         <v>1132</v>
       </c>
       <c r="E1143">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F1143" t="s">
         <v>914</v>
@@ -56977,7 +56976,7 @@
         <v>1132</v>
       </c>
       <c r="E1144">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F1144" t="s">
         <v>914</v>
@@ -57009,7 +57008,7 @@
         <v>1132</v>
       </c>
       <c r="E1145">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F1145" t="s">
         <v>914</v>
@@ -57041,7 +57040,7 @@
         <v>1132</v>
       </c>
       <c r="E1146">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F1146" t="s">
         <v>914</v>
@@ -57073,7 +57072,7 @@
         <v>1132</v>
       </c>
       <c r="E1147">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F1147" t="s">
         <v>914</v>
@@ -57139,7 +57138,7 @@
         <v>1132</v>
       </c>
       <c r="E1150">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F1150" t="s">
         <v>914</v>
@@ -57171,7 +57170,7 @@
         <v>1132</v>
       </c>
       <c r="E1151">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F1151" t="s">
         <v>914</v>
@@ -57203,7 +57202,7 @@
         <v>1132</v>
       </c>
       <c r="E1152">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1152" t="s">
         <v>914</v>
@@ -57235,7 +57234,7 @@
         <v>1132</v>
       </c>
       <c r="E1153">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F1153" t="s">
         <v>914</v>
@@ -57267,7 +57266,7 @@
         <v>1132</v>
       </c>
       <c r="E1154">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F1154" t="s">
         <v>914</v>
@@ -57299,7 +57298,7 @@
         <v>1132</v>
       </c>
       <c r="E1155">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F1155" t="s">
         <v>914</v>
@@ -57331,7 +57330,7 @@
         <v>1132</v>
       </c>
       <c r="E1156">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F1156" t="s">
         <v>914</v>
@@ -57363,7 +57362,7 @@
         <v>1132</v>
       </c>
       <c r="E1157">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F1157" t="s">
         <v>914</v>
@@ -57395,7 +57394,7 @@
         <v>1132</v>
       </c>
       <c r="E1158">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1158" t="s">
         <v>914</v>
@@ -57427,7 +57426,7 @@
         <v>1132</v>
       </c>
       <c r="E1159">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1159" t="s">
         <v>914</v>
@@ -57459,7 +57458,7 @@
         <v>1132</v>
       </c>
       <c r="E1160">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1160" t="s">
         <v>914</v>
@@ -57491,7 +57490,7 @@
         <v>1132</v>
       </c>
       <c r="E1161">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F1161" t="s">
         <v>914</v>
@@ -57543,10 +57542,10 @@
       <c r="A4" s="3" t="s">
         <v>991</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4">
         <v>746</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4">
         <v>746</v>
       </c>
     </row>
@@ -57554,10 +57553,10 @@
       <c r="A5" s="3" t="s">
         <v>992</v>
       </c>
-      <c r="B5" s="5">
+      <c r="B5">
         <v>1</v>
       </c>
-      <c r="C5" s="5">
+      <c r="C5">
         <v>1</v>
       </c>
     </row>
@@ -57565,10 +57564,10 @@
       <c r="A6" s="3" t="s">
         <v>990</v>
       </c>
-      <c r="B6" s="5">
+      <c r="B6">
         <v>150</v>
       </c>
-      <c r="C6" s="5">
+      <c r="C6">
         <v>152</v>
       </c>
     </row>
@@ -57576,10 +57575,10 @@
       <c r="A7" s="3" t="s">
         <v>1145</v>
       </c>
-      <c r="B7" s="5">
+      <c r="B7">
         <v>5</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C7">
         <v>5</v>
       </c>
     </row>
@@ -57587,10 +57586,10 @@
       <c r="A8" s="3" t="s">
         <v>1409</v>
       </c>
-      <c r="B8" s="5">
+      <c r="B8">
         <v>248</v>
       </c>
-      <c r="C8" s="5">
+      <c r="C8">
         <v>256</v>
       </c>
     </row>
@@ -57598,10 +57597,10 @@
       <c r="A9" s="3" t="s">
         <v>989</v>
       </c>
-      <c r="B9" s="5">
+      <c r="B9">
         <v>1150</v>
       </c>
-      <c r="C9" s="5">
+      <c r="C9">
         <v>1160</v>
       </c>
     </row>

</xml_diff>